<commit_message>
fix: quadsim bugs; remade Unity env to be more realistic
</commit_message>
<xml_diff>
--- a/5 - Experimental Data/july_14_2026_water_bottle/July 14 2026 Results.xlsx
+++ b/5 - Experimental Data/july_14_2026_water_bottle/July 14 2026 Results.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/max/Documents/GitHub/rise-controller/5 - Experimental Data/july_14_2026_water_bottle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B9ADDC0-2611-9B45-86AE-4030EA84BD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4103099-1243-AE4A-A6E4-563D0A09702C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="24040" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Controls Experiment Results" sheetId="1" r:id="rId1"/>
+    <sheet name="July 14" sheetId="1" r:id="rId1"/>
+    <sheet name="Summaries" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
   <si>
     <t>Controller</t>
   </si>
@@ -108,13 +109,16 @@
   </si>
   <si>
     <t>NoResNet (Baseline)</t>
+  </si>
+  <si>
+    <t>Date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -131,6 +135,13 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -156,11 +167,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -379,7 +393,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
@@ -392,10 +406,10 @@
     <col min="8" max="8" width="4.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
     <col min="14" max="14" width="14.33203125" customWidth="1"/>
-    <col min="15" max="15" width="55.1640625" customWidth="1"/>
+    <col min="16" max="16" width="55.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -439,10 +453,13 @@
         <v>21</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -488,8 +505,11 @@
       <c r="N2" s="1">
         <v>1.5347</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="O2" s="5">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -535,8 +555,11 @@
       <c r="N3" s="1">
         <v>1.3765000000000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="O3" s="5">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -582,8 +605,11 @@
       <c r="N4" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="O4" s="5">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -629,8 +655,11 @@
       <c r="N5" s="1">
         <v>2.11</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="O5" s="5">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -676,8 +705,11 @@
       <c r="N6" s="1">
         <v>1.8535999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="O6" s="5">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -723,11 +755,14 @@
       <c r="N7" s="1">
         <v>1.9803999999999999</v>
       </c>
-      <c r="O7" s="1" t="s">
+      <c r="O7" s="5">
+        <v>46217</v>
+      </c>
+      <c r="P7" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -773,8 +808,11 @@
       <c r="N8" s="1">
         <v>1.8149999999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="O8" s="5">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -820,105 +858,240 @@
       <c r="N9" s="1">
         <v>2.0699999999999998</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="1" t="s">
+      <c r="O9" s="5">
+        <v>46217</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A001CB-0E61-0544-B3B1-F07FB7C13439}">
+  <dimension ref="A1:P10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A1" s="6">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="1" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B3" s="4">
         <v>0.109</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C3" s="4">
         <v>1.5347</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="1" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B4" s="4">
         <v>0.11550000000000001</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C4" s="4">
         <v>1.3765000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="1" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B5" s="4">
         <v>0.13400000000000001</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="1" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B6" s="4">
         <v>0.1414</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C6" s="4">
         <v>2.11</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="1" t="s">
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B7" s="4">
         <v>0.14319999999999999</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C7" s="4">
         <v>1.8535999999999999</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="1" t="s">
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B8" s="4">
         <v>8.7099999999999997E-2</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C8" s="4">
         <v>1.9803999999999999</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="1" t="s">
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B9" s="4">
         <v>9.0399999999999994E-2</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C9" s="4">
         <v>1.8149999999999999</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="1" t="s">
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B10" s="4">
         <v>8.5199999999999998E-2</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C10" s="4">
         <v>2.0699999999999998</v>
       </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
renamed stuff. Preparing for real-world experiment
</commit_message>
<xml_diff>
--- a/5 - Experimental Data/july_14_2026_water_bottle/July 14 2026 Results.xlsx
+++ b/5 - Experimental Data/july_14_2026_water_bottle/July 14 2026 Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/max/Documents/GitHub/rise-controller/5 - Experimental Data/july_14_2026_water_bottle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4103099-1243-AE4A-A6E4-563D0A09702C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5578C68-963D-B547-AEF5-CE0004DFBFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="24040" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
   <si>
     <t>Controller</t>
   </si>
@@ -75,9 +75,6 @@
     <t>IntegratedResNet</t>
   </si>
   <si>
-    <t>NoResNet</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
@@ -112,6 +109,12 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Baseline</t>
+  </si>
+  <si>
+    <t>Cristian gains</t>
   </si>
 </sst>
 </file>
@@ -147,12 +150,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -167,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -175,6 +184,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,14 +403,12 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.1640625" customWidth="1"/>
-    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.1640625" customWidth="1"/>
-    <col min="5" max="5" width="3.6640625" customWidth="1"/>
+    <col min="3" max="5" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.1640625" customWidth="1"/>
     <col min="7" max="7" width="7.6640625" customWidth="1"/>
     <col min="8" max="8" width="4.6640625" bestFit="1" customWidth="1"/>
@@ -414,7 +422,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -447,13 +455,13 @@
         <v>10</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="O1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>11</v>
@@ -476,15 +484,15 @@
         <v>2.4</v>
       </c>
       <c r="F2" s="2">
-        <f t="shared" ref="F2:F9" si="0">C2*D2+D2*E2+C2*E2+1</f>
+        <f t="shared" ref="F2:F10" si="0">C2*D2+D2*E2+C2*E2+1</f>
         <v>3.0712000000000002</v>
       </c>
       <c r="G2" s="2">
-        <f t="shared" ref="G2:G9" si="1">C2*D2*E2+C2</f>
+        <f t="shared" ref="G2:G10" si="1">C2*D2*E2+C2</f>
         <v>0.91008</v>
       </c>
       <c r="H2" s="2">
-        <f t="shared" ref="H2:H9" si="2">C2+D2+E2</f>
+        <f t="shared" ref="H2:H10" si="2">C2+D2+E2</f>
         <v>3.23</v>
       </c>
       <c r="I2" s="1">
@@ -561,10 +569,10 @@
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1">
         <v>0.72</v>
@@ -591,10 +599,10 @@
         <v>0.5</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L4" s="1">
         <v>54.294499999999999</v>
@@ -603,7 +611,7 @@
         <v>0.13400000000000001</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O4" s="5">
         <v>46217</v>
@@ -611,7 +619,7 @@
     </row>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1">
         <v>2</v>
@@ -641,10 +649,10 @@
         <v>0.01</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L5" s="1">
         <v>67</v>
@@ -661,7 +669,7 @@
     </row>
     <row r="6" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
@@ -691,10 +699,10 @@
         <v>0.5</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L6" s="1">
         <v>60.08</v>
@@ -711,7 +719,7 @@
     </row>
     <row r="7" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
@@ -759,12 +767,12 @@
         <v>46217</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="1">
         <v>3</v>
@@ -814,7 +822,7 @@
     </row>
     <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="1">
         <v>2</v>
@@ -861,6 +869,189 @@
       <c r="O9" s="5">
         <v>46217</v>
       </c>
+    </row>
+    <row r="10" spans="1:16" s="7" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="F11" s="2">
+        <f>C11*D11+D11*E11+C11*E11+1</f>
+        <v>9.625</v>
+      </c>
+      <c r="G11" s="2">
+        <f>C11*D11*E11+C11</f>
+        <v>5.375</v>
+      </c>
+      <c r="H11" s="2">
+        <f>C11+D11+E11</f>
+        <v>5.25</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+    </row>
+    <row r="25" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+    </row>
+    <row r="26" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+    </row>
+    <row r="30" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+    </row>
+    <row r="33" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+    </row>
+    <row r="35" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+    </row>
+    <row r="36" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+    </row>
+    <row r="37" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+    </row>
+    <row r="38" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+    </row>
+    <row r="39" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+    </row>
+    <row r="40" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" spans="6:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -882,10 +1073,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -903,7 +1094,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="4">
         <v>0.109</v>
@@ -927,7 +1118,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="4">
         <v>0.11550000000000001</v>
@@ -951,13 +1142,13 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A5" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B5" s="4">
         <v>0.13400000000000001</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -975,7 +1166,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A6" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="4">
         <v>0.1414</v>
@@ -999,7 +1190,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="4">
         <v>0.14319999999999999</v>
@@ -1023,7 +1214,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A8" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="4">
         <v>8.7099999999999997E-2</v>
@@ -1047,7 +1238,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="4">
         <v>9.0399999999999994E-2</v>
@@ -1071,7 +1262,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A10" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" s="4">
         <v>8.5199999999999998E-2</v>

</xml_diff>